<commit_message>
🗂 Folletos 2026-05 generados automáticamente
</commit_message>
<xml_diff>
--- a/inputs/templates/TEMPLATE_FONDO_LIQUIDEZ_ACTIVA.xlsx
+++ b/inputs/templates/TEMPLATE_FONDO_LIQUIDEZ_ACTIVA.xlsx
@@ -26,7 +26,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="9">
+  <numFmts count="10">
     <numFmt numFmtId="164" formatCode="#,##0.0000"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
     <numFmt numFmtId="166" formatCode="m/d/yyyy"/>
@@ -36,6 +36,7 @@
     <numFmt numFmtId="170" formatCode="_ * #,##0.000_ ;_ * \-#,##0.000_ ;_ * \-_ ;_ @_ "/>
     <numFmt numFmtId="171" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * \-_ ;_ @_ "/>
     <numFmt numFmtId="172" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
+    <numFmt numFmtId="173" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="30">
     <font>
@@ -335,7 +336,7 @@
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="178">
+  <cellXfs count="179">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -868,6 +869,7 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
+    <xf numFmtId="173" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="11">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2481,7 +2483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:BK247"/>
+  <dimension ref="A1:BK499"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.2890625" defaultRowHeight="13.5" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14.14" customWidth="1" style="92" min="1" max="1"/>
@@ -4834,7 +4836,7 @@
         </is>
       </c>
       <c r="AW19" s="118" t="n">
-        <v>46142</v>
+        <v>46144</v>
       </c>
       <c r="AX19" s="119">
         <f>EOMONTH($AW19,AX18)</f>
@@ -18143,7 +18145,48 @@
         <v/>
       </c>
     </row>
-    <row r="248" ht="13.5" customHeight="1" s="90"/>
+    <row r="248" ht="13.5" customHeight="1" s="90">
+      <c r="A248" s="178" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B248" t="n">
+        <v>19991.53842678169</v>
+      </c>
+      <c r="C248">
+        <f>(B248/B247-1)/(A248-A247)*30</f>
+        <v/>
+      </c>
+      <c r="D248">
+        <f>B248/$B$3*100</f>
+        <v/>
+      </c>
+      <c r="F248" s="178" t="n">
+        <v>46144</v>
+      </c>
+      <c r="G248" t="n">
+        <v>1070.9923</v>
+      </c>
+      <c r="H248">
+        <f>+G248+$S$146+$S$148+$S$150+$S$152+$S$154+$S$156+$S$158+$S$160+$S$162</f>
+        <v/>
+      </c>
+      <c r="I248">
+        <f>+(H248/H247-1)/(F248-F247)*30</f>
+        <v/>
+      </c>
+      <c r="J248">
+        <f>+J247*(1+I248)</f>
+        <v/>
+      </c>
+      <c r="L248">
+        <f>+(K248/K247-1)/(F248-F247)*30</f>
+        <v/>
+      </c>
+      <c r="M248">
+        <f>+M247*(1+L248)</f>
+        <v/>
+      </c>
+    </row>
     <row r="249" ht="13.5" customHeight="1" s="90"/>
     <row r="250" ht="13.5" customHeight="1" s="90"/>
     <row r="251" ht="13.5" customHeight="1" s="90"/>
@@ -18171,6 +18214,230 @@
     <row r="273" ht="13.5" customHeight="1" s="90"/>
     <row r="274" ht="13.5" customHeight="1" s="90"/>
     <row r="275" ht="13.5" customHeight="1" s="90"/>
+    <row r="276"/>
+    <row r="277"/>
+    <row r="278"/>
+    <row r="279"/>
+    <row r="280"/>
+    <row r="281"/>
+    <row r="282"/>
+    <row r="283"/>
+    <row r="284"/>
+    <row r="285"/>
+    <row r="286"/>
+    <row r="287"/>
+    <row r="288"/>
+    <row r="289"/>
+    <row r="290"/>
+    <row r="291"/>
+    <row r="292"/>
+    <row r="293"/>
+    <row r="294"/>
+    <row r="295"/>
+    <row r="296"/>
+    <row r="297"/>
+    <row r="298"/>
+    <row r="299"/>
+    <row r="300"/>
+    <row r="301"/>
+    <row r="302"/>
+    <row r="303"/>
+    <row r="304"/>
+    <row r="305"/>
+    <row r="306"/>
+    <row r="307"/>
+    <row r="308"/>
+    <row r="309"/>
+    <row r="310"/>
+    <row r="311"/>
+    <row r="312"/>
+    <row r="313"/>
+    <row r="314"/>
+    <row r="315"/>
+    <row r="316"/>
+    <row r="317"/>
+    <row r="318"/>
+    <row r="319"/>
+    <row r="320"/>
+    <row r="321"/>
+    <row r="322"/>
+    <row r="323"/>
+    <row r="324"/>
+    <row r="325"/>
+    <row r="326"/>
+    <row r="327"/>
+    <row r="328"/>
+    <row r="329"/>
+    <row r="330"/>
+    <row r="331"/>
+    <row r="332"/>
+    <row r="333"/>
+    <row r="334"/>
+    <row r="335"/>
+    <row r="336"/>
+    <row r="337"/>
+    <row r="338"/>
+    <row r="339"/>
+    <row r="340"/>
+    <row r="341"/>
+    <row r="342"/>
+    <row r="343"/>
+    <row r="344"/>
+    <row r="345"/>
+    <row r="346"/>
+    <row r="347"/>
+    <row r="348"/>
+    <row r="349"/>
+    <row r="350"/>
+    <row r="351"/>
+    <row r="352"/>
+    <row r="353"/>
+    <row r="354"/>
+    <row r="355"/>
+    <row r="356"/>
+    <row r="357"/>
+    <row r="358"/>
+    <row r="359"/>
+    <row r="360"/>
+    <row r="361"/>
+    <row r="362"/>
+    <row r="363"/>
+    <row r="364"/>
+    <row r="365"/>
+    <row r="366"/>
+    <row r="367"/>
+    <row r="368"/>
+    <row r="369"/>
+    <row r="370"/>
+    <row r="371"/>
+    <row r="372"/>
+    <row r="373"/>
+    <row r="374"/>
+    <row r="375"/>
+    <row r="376"/>
+    <row r="377"/>
+    <row r="378"/>
+    <row r="379"/>
+    <row r="380"/>
+    <row r="381"/>
+    <row r="382"/>
+    <row r="383"/>
+    <row r="384"/>
+    <row r="385"/>
+    <row r="386"/>
+    <row r="387"/>
+    <row r="388"/>
+    <row r="389"/>
+    <row r="390"/>
+    <row r="391"/>
+    <row r="392"/>
+    <row r="393"/>
+    <row r="394"/>
+    <row r="395"/>
+    <row r="396"/>
+    <row r="397"/>
+    <row r="398"/>
+    <row r="399"/>
+    <row r="400"/>
+    <row r="401"/>
+    <row r="402"/>
+    <row r="403"/>
+    <row r="404"/>
+    <row r="405"/>
+    <row r="406"/>
+    <row r="407"/>
+    <row r="408"/>
+    <row r="409"/>
+    <row r="410"/>
+    <row r="411"/>
+    <row r="412"/>
+    <row r="413"/>
+    <row r="414"/>
+    <row r="415"/>
+    <row r="416"/>
+    <row r="417"/>
+    <row r="418"/>
+    <row r="419"/>
+    <row r="420"/>
+    <row r="421"/>
+    <row r="422"/>
+    <row r="423"/>
+    <row r="424"/>
+    <row r="425"/>
+    <row r="426"/>
+    <row r="427"/>
+    <row r="428"/>
+    <row r="429"/>
+    <row r="430"/>
+    <row r="431"/>
+    <row r="432"/>
+    <row r="433"/>
+    <row r="434"/>
+    <row r="435"/>
+    <row r="436"/>
+    <row r="437"/>
+    <row r="438"/>
+    <row r="439"/>
+    <row r="440"/>
+    <row r="441"/>
+    <row r="442"/>
+    <row r="443"/>
+    <row r="444"/>
+    <row r="445"/>
+    <row r="446"/>
+    <row r="447"/>
+    <row r="448"/>
+    <row r="449"/>
+    <row r="450"/>
+    <row r="451"/>
+    <row r="452"/>
+    <row r="453"/>
+    <row r="454"/>
+    <row r="455"/>
+    <row r="456"/>
+    <row r="457"/>
+    <row r="458"/>
+    <row r="459"/>
+    <row r="460"/>
+    <row r="461"/>
+    <row r="462"/>
+    <row r="463"/>
+    <row r="464"/>
+    <row r="465"/>
+    <row r="466"/>
+    <row r="467"/>
+    <row r="468"/>
+    <row r="469"/>
+    <row r="470"/>
+    <row r="471"/>
+    <row r="472"/>
+    <row r="473"/>
+    <row r="474"/>
+    <row r="475"/>
+    <row r="476"/>
+    <row r="477"/>
+    <row r="478"/>
+    <row r="479"/>
+    <row r="480"/>
+    <row r="481"/>
+    <row r="482"/>
+    <row r="483"/>
+    <row r="484"/>
+    <row r="485"/>
+    <row r="486"/>
+    <row r="487"/>
+    <row r="488"/>
+    <row r="489"/>
+    <row r="490"/>
+    <row r="491"/>
+    <row r="492"/>
+    <row r="493"/>
+    <row r="494"/>
+    <row r="495"/>
+    <row r="496"/>
+    <row r="497"/>
+    <row r="498"/>
+    <row r="499"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="AV28:AV29"/>

</xml_diff>